<commit_message>
Updated Description, Outcome Message, Sensitivity, Groupiing Variable QNAM and negative test.
</commit_message>
<xml_diff>
--- a/rules/CORE-000533/negative/01/data/unit-test-coreid-CG0138-negative.xlsx
+++ b/rules/CORE-000533/negative/01/data/unit-test-coreid-CG0138-negative.xlsx
@@ -36,7 +36,7 @@
       <i val="1"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -53,6 +53,11 @@
       <patternFill patternType="solid">
         <fgColor theme="0" tint="-0.1499984740745262"/>
         <bgColor theme="0" tint="-0.1499984740745262"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
       </patternFill>
     </fill>
   </fills>
@@ -83,7 +88,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -110,6 +115,10 @@
     <xf numFmtId="49" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -563,7 +572,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -595,6 +604,62 @@
       <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Error value</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>suppec.xpt</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>7</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>QNAM</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>SAFETY</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>suppec.xpt</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>8</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>QNAM</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>ITT</t>
         </is>
       </c>
     </row>
@@ -971,7 +1036,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J7"/>
+  <dimension ref="A1:J8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1292,7 +1357,7 @@
           <t>124</t>
         </is>
       </c>
-      <c r="F7" s="4" t="inlineStr">
+      <c r="F7" s="10" t="inlineStr">
         <is>
           <t>SAFETY</t>
         </is>
@@ -1313,6 +1378,58 @@
         </is>
       </c>
       <c r="J7" s="4" t="inlineStr">
+        <is>
+          <t>INVESTIGATOR</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>CDISCPILOT01</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>EC</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>CDISC009</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>ECSEQ</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>125</t>
+        </is>
+      </c>
+      <c r="F8" s="11" t="inlineStr">
+        <is>
+          <t>ITT</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Intent-To-Treat Flag</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>COLLECTED</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
         <is>
           <t>INVESTIGATOR</t>
         </is>

</xml_diff>